<commit_message>
feat: sync database with excel inventory, lock zone to Caracas el Este and embed product images
</commit_message>
<xml_diff>
--- a/frontend/public/data/productos_inventario.xlsx
+++ b/frontend/public/data/productos_inventario.xlsx
@@ -2502,7 +2502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2511,10 +2511,11 @@
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2550,20 +2551,25 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Imagen (Archivo)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Etiquetas</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Stock Almacén</t>
         </is>
@@ -2598,15 +2604,20 @@
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>tomates_perita.png</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="n">
-        <v>58</v>
-      </c>
+      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
-        <v>196</v>
+        <v>18</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>388</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
@@ -2638,15 +2649,20 @@
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>cebolla_blanca.png</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="n">
-        <v>21</v>
-      </c>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="n">
-        <v>221</v>
+        <v>39</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>163</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
@@ -2678,15 +2694,20 @@
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>papa_lavada.png</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="n">
-        <v>53</v>
-      </c>
+      <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="n">
-        <v>127</v>
+        <v>14</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>315</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
@@ -2718,15 +2739,20 @@
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>zanahoria.png</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="n">
-        <v>55</v>
-      </c>
+      <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="n">
-        <v>308</v>
+        <v>73</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>477</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
@@ -2758,19 +2784,20 @@
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>pimenton_verde.png</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>51</v>
-      </c>
+      <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="n">
-        <v>367</v>
+        <v>44</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>427</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
@@ -2802,15 +2829,24 @@
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
+          <t>lechuga_romana.png</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="n">
-        <v>91</v>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>194</v>
+        <v>18</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>344</v>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
@@ -2842,19 +2878,20 @@
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>platano_maduro.png</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>42</v>
-      </c>
+      <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n">
-        <v>495</v>
+        <v>13</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
@@ -2886,15 +2923,20 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
+          <t>cambur.png</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="n">
-        <v>58</v>
-      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n">
-        <v>396</v>
+        <v>31</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>321</v>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
@@ -2926,15 +2968,20 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
+          <t>manzana_gala.png</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="n">
-        <v>40</v>
-      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
-        <v>349</v>
+        <v>54</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>310</v>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
@@ -2966,15 +3013,20 @@
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
+          <t>naranja.png</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="n">
-        <v>53</v>
-      </c>
+      <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
-        <v>202</v>
+        <v>35</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>408</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
@@ -3006,15 +3058,20 @@
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
+          <t>lechosa.png</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="n">
-        <v>71</v>
+        <v>43</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>199</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
@@ -3046,15 +3103,20 @@
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
+          <t>limones.png</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="n">
-        <v>100</v>
-      </c>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="n">
-        <v>74</v>
+        <v>61</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>361</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
@@ -3086,19 +3148,20 @@
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
+          <t>pina.png</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>39</v>
-      </c>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="n">
-        <v>405</v>
+        <v>98</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>387</v>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
@@ -3130,15 +3193,20 @@
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
+          <t>aguacate.png</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="n">
-        <v>52</v>
-      </c>
+      <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="n">
-        <v>172</v>
+        <v>24</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>370</v>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
@@ -3170,15 +3238,24 @@
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
+          <t>frutas_picadas.png</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
           <t>500g</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="n">
-        <v>75</v>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>62</v>
+        <v>52</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>240</v>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
@@ -3210,15 +3287,20 @@
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
+          <t>carne_molida.png</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="n">
-        <v>43</v>
-      </c>
+      <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="n">
-        <v>477</v>
+        <v>67</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>256</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
@@ -3250,19 +3332,20 @@
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
+          <t>bistec_ganso.png</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>76</v>
-      </c>
+      <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="n">
-        <v>271</v>
+        <v>40</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>366</v>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
@@ -3294,15 +3377,20 @@
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
+          <t>costilla_res.png</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="n">
-        <v>73</v>
-      </c>
+      <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n">
-        <v>137</v>
+        <v>37</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>493</v>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
@@ -3334,15 +3422,24 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
+          <t>pechuga_pollo.png</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="n">
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
         <v>91</v>
       </c>
-      <c r="J20" s="2" t="n">
-        <v>316</v>
+      <c r="K20" s="2" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
@@ -3374,15 +3471,24 @@
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
+          <t>pollo_entero.png</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="n">
-        <v>95</v>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>277</v>
+        <v>48</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>274</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
@@ -3414,15 +3520,20 @@
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
+          <t>muslos_pollo.png</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="n">
-        <v>66</v>
-      </c>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n">
-        <v>492</v>
+        <v>50</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>292</v>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
@@ -3454,15 +3565,20 @@
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
+          <t>alitas_pollo.png</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="n">
-        <v>87</v>
-      </c>
+      <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="n">
-        <v>309</v>
+        <v>95</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1">
@@ -3494,15 +3610,20 @@
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
+          <t>jamon_cocido.png</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
           <t>500g</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="n">
-        <v>14</v>
-      </c>
+      <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="n">
-        <v>287</v>
+        <v>67</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>469</v>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -3534,15 +3655,20 @@
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
+          <t>queso_amarillo.png</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
           <t>500g</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="n">
-        <v>89</v>
-      </c>
+      <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="n">
-        <v>107</v>
+        <v>63</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>289</v>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
@@ -3574,15 +3700,20 @@
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
+          <t>queso_blanco.png</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="n">
-        <v>26</v>
-      </c>
+      <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="n">
-        <v>53</v>
+        <v>67</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>499</v>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
@@ -3614,15 +3745,20 @@
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
+          <t>salchichas.png</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
           <t>1 Paquete</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="n">
-        <v>85</v>
-      </c>
+      <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="n">
-        <v>258</v>
+        <v>89</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>351</v>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
@@ -3654,15 +3790,20 @@
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
+          <t>tocino.png</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
           <t>250g</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="n">
-        <v>34</v>
-      </c>
+      <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="n">
-        <v>86</v>
+        <v>20</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>253</v>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
@@ -3694,15 +3835,20 @@
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
+          <t>chorizo.png</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
           <t>500g</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="n">
-        <v>17</v>
-      </c>
+      <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="n">
-        <v>136</v>
+        <v>88</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>313</v>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
@@ -3734,15 +3880,24 @@
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
+          <t>queso_guayanes.png</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
           <t>500g</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="n">
-        <v>15</v>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>443</v>
+        <v>77</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>315</v>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
@@ -3774,15 +3929,24 @@
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
+          <t>nuggets.png</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
           <t>1 Paquete</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="n">
-        <v>61</v>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J31" s="2" t="n">
-        <v>425</v>
+        <v>75</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>161</v>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
@@ -3814,15 +3978,20 @@
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
+          <t>coca_cola.png</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
           <t>2 L</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="n">
-        <v>32</v>
-      </c>
+      <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="n">
-        <v>368</v>
+        <v>71</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -3854,15 +4023,20 @@
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
+          <t>pepsi.png</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
           <t>2 L</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="n">
-        <v>41</v>
-      </c>
+      <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="n">
-        <v>286</v>
+        <v>52</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>441</v>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
@@ -3894,15 +4068,24 @@
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
+          <t>chinotto.png</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
           <t>2 L</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="n">
-        <v>33</v>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>165</v>
+        <v>77</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>208</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
@@ -3934,19 +4117,20 @@
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
+          <t>frescolita.png</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
           <t>2 L</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="n">
-        <v>20</v>
-      </c>
+      <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="n">
-        <v>229</v>
+        <v>48</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>487</v>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
@@ -3978,15 +4162,20 @@
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
+          <t>maltin.png</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
           <t>1.5 L</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="n">
-        <v>16</v>
-      </c>
+      <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="n">
-        <v>283</v>
+        <v>92</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>182</v>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
@@ -4018,15 +4207,24 @@
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
+          <t>arroz_blanco.png</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="2" t="n">
-        <v>62</v>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J37" s="2" t="n">
-        <v>375</v>
+        <v>57</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>354</v>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
@@ -4058,15 +4256,20 @@
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
+          <t>arroz_primor.png</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="n">
-        <v>46</v>
-      </c>
+      <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="n">
-        <v>374</v>
+        <v>57</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>203</v>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
@@ -4098,15 +4301,20 @@
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
+          <t>pasta_capri.png</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="n">
-        <v>62</v>
-      </c>
+      <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="n">
-        <v>330</v>
+        <v>16</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
@@ -4138,15 +4346,24 @@
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
+          <t>harina_pan.png</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="n">
-        <v>79</v>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>455</v>
+        <v>23</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>338</v>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
@@ -4178,15 +4395,20 @@
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
+          <t>caraotas.png</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
           <t>500g</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="2" t="n">
-        <v>35</v>
-      </c>
+      <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="n">
-        <v>242</v>
+        <v>98</v>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>168</v>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
@@ -4218,15 +4440,24 @@
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
+          <t>lentejas.png</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
           <t>500g</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="n">
-        <v>49</v>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J42" s="2" t="n">
-        <v>84</v>
+        <v>70</v>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>349</v>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
@@ -4258,15 +4489,20 @@
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
+          <t>atun_aceite.png</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
           <t>140g</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="2" t="n">
-        <v>80</v>
-      </c>
+      <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="n">
-        <v>206</v>
+        <v>44</v>
+      </c>
+      <c r="K43" s="2" t="n">
+        <v>355</v>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
@@ -4298,15 +4534,20 @@
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
+          <t>atun_agua.png</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
           <t>140g</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="n">
-        <v>71</v>
-      </c>
+      <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="n">
-        <v>153</v>
+        <v>77</v>
+      </c>
+      <c r="K44" s="2" t="n">
+        <v>294</v>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
@@ -4338,19 +4579,24 @@
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
+          <t>maiz_lata.png</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
           <t>300g</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="n">
-        <v>60</v>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J45" s="2" t="n">
-        <v>167</v>
+        <v>96</v>
+      </c>
+      <c r="K45" s="2" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="46" ht="60" customHeight="1">
@@ -4382,15 +4628,20 @@
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
+          <t>aceite_maiz.png</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
           <t>1 Litro</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="n">
-        <v>64</v>
-      </c>
+      <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="n">
-        <v>343</v>
+        <v>98</v>
+      </c>
+      <c r="K46" s="2" t="n">
+        <v>252</v>
       </c>
     </row>
     <row r="47" ht="60" customHeight="1">
@@ -4422,15 +4673,20 @@
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
+          <t>jabon_protex.png</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
           <t>3 Unidades</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="n">
-        <v>26</v>
-      </c>
+      <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="n">
-        <v>467</v>
+        <v>50</v>
+      </c>
+      <c r="K47" s="2" t="n">
+        <v>176</v>
       </c>
     </row>
     <row r="48" ht="60" customHeight="1">
@@ -4462,15 +4718,24 @@
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
+          <t>desodorante.png</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
           <t>50ml</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="n">
-        <v>90</v>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>343</v>
+        <v>65</v>
+      </c>
+      <c r="K48" s="2" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
@@ -4502,15 +4767,20 @@
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
+          <t>crema_dental.png</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
           <t>100g</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr"/>
-      <c r="I49" s="2" t="n">
-        <v>88</v>
-      </c>
+      <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="n">
-        <v>114</v>
+        <v>21</v>
+      </c>
+      <c r="K49" s="2" t="n">
+        <v>143</v>
       </c>
     </row>
     <row r="50" ht="60" customHeight="1">
@@ -4542,15 +4812,20 @@
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
+          <t>shampoo.png</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
           <t>400ml</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="n">
-        <v>93</v>
-      </c>
+      <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="n">
-        <v>389</v>
+        <v>92</v>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>204</v>
       </c>
     </row>
     <row r="51" ht="60" customHeight="1">
@@ -4582,19 +4857,20 @@
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
+          <t>papel_higienico.png</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
           <t>4 Rollos</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="I51" s="2" t="n">
-        <v>85</v>
-      </c>
+      <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="n">
-        <v>301</v>
+        <v>51</v>
+      </c>
+      <c r="K51" s="2" t="n">
+        <v>138</v>
       </c>
     </row>
     <row r="52" ht="60" customHeight="1">
@@ -4626,15 +4902,20 @@
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
+          <t>toallas_sanitarias.png</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
           <t>10 Unidades</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="n">
-        <v>69</v>
-      </c>
+      <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="n">
-        <v>63</v>
+        <v>82</v>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>312</v>
       </c>
     </row>
     <row r="53" ht="60" customHeight="1">
@@ -4666,19 +4947,20 @@
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
+          <t>maquina_afeitar.png</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
           <t>2 Unidades</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="n">
-        <v>14</v>
-      </c>
+      <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="n">
-        <v>362</v>
+        <v>70</v>
+      </c>
+      <c r="K53" s="2" t="n">
+        <v>380</v>
       </c>
     </row>
     <row r="54" ht="60" customHeight="1">
@@ -4710,15 +4992,20 @@
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
+          <t>crema_corporal.png</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
           <t>400ml</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="n">
-        <v>38</v>
-      </c>
+      <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="n">
-        <v>396</v>
+        <v>34</v>
+      </c>
+      <c r="K54" s="2" t="n">
+        <v>268</v>
       </c>
     </row>
     <row r="55" ht="60" customHeight="1">
@@ -4750,15 +5037,20 @@
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
+          <t>algodon.png</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
           <t>100g</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr"/>
-      <c r="I55" s="2" t="n">
-        <v>32</v>
-      </c>
+      <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="n">
-        <v>107</v>
+        <v>100</v>
+      </c>
+      <c r="K55" s="2" t="n">
+        <v>411</v>
       </c>
     </row>
     <row r="56" ht="60" customHeight="1">
@@ -4790,15 +5082,20 @@
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
+          <t>hisopos.png</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
           <t>100 Unidades</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="2" t="n">
-        <v>68</v>
-      </c>
+      <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="n">
-        <v>293</v>
+        <v>19</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>374</v>
       </c>
     </row>
     <row r="57" ht="60" customHeight="1">
@@ -4830,15 +5127,24 @@
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
+          <t>alcohol.png</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
           <t>250ml</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr"/>
-      <c r="I57" s="2" t="n">
-        <v>30</v>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J57" s="2" t="n">
-        <v>290</v>
+        <v>92</v>
+      </c>
+      <c r="K57" s="2" t="n">
+        <v>107</v>
       </c>
     </row>
     <row r="58" ht="60" customHeight="1">
@@ -4870,15 +5176,20 @@
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
+          <t>agua_oxigenada.png</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
           <t>100ml</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr"/>
-      <c r="I58" s="2" t="n">
-        <v>17</v>
-      </c>
+      <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="n">
-        <v>311</v>
+        <v>94</v>
+      </c>
+      <c r="K58" s="2" t="n">
+        <v>422</v>
       </c>
     </row>
     <row r="59" ht="60" customHeight="1">
@@ -4910,15 +5221,20 @@
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
+          <t>curitas.png</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
           <t>Caja</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr"/>
-      <c r="I59" s="2" t="n">
-        <v>90</v>
-      </c>
+      <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="n">
-        <v>166</v>
+        <v>70</v>
+      </c>
+      <c r="K59" s="2" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="60" ht="60" customHeight="1">
@@ -4950,15 +5266,24 @@
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
+          <t>detergente_liquido.png</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
           <t>2 L</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="2" t="n">
-        <v>96</v>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J60" s="2" t="n">
-        <v>452</v>
+        <v>76</v>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="61" ht="60" customHeight="1">
@@ -4990,15 +5315,24 @@
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
+          <t>detergente_polvo.png</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr"/>
-      <c r="I61" s="2" t="n">
-        <v>26</v>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J61" s="2" t="n">
-        <v>220</v>
+        <v>75</v>
+      </c>
+      <c r="K61" s="2" t="n">
+        <v>459</v>
       </c>
     </row>
     <row r="62" ht="60" customHeight="1">
@@ -5030,15 +5364,20 @@
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
+          <t>suavizante.png</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
           <t>1 L</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr"/>
-      <c r="I62" s="2" t="n">
-        <v>28</v>
-      </c>
+      <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="n">
-        <v>57</v>
+        <v>60</v>
+      </c>
+      <c r="K62" s="2" t="n">
+        <v>93</v>
       </c>
     </row>
     <row r="63" ht="60" customHeight="1">
@@ -5070,15 +5409,20 @@
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
+          <t>lavaplatos_liquido.png</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
           <t>500ml</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr"/>
-      <c r="I63" s="2" t="n">
-        <v>74</v>
-      </c>
+      <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="n">
-        <v>58</v>
+        <v>96</v>
+      </c>
+      <c r="K63" s="2" t="n">
+        <v>369</v>
       </c>
     </row>
     <row r="64" ht="60" customHeight="1">
@@ -5110,15 +5454,20 @@
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
+          <t>lavaplatos_crema.png</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
           <t>250g</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="2" t="n">
-        <v>73</v>
-      </c>
+      <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="n">
-        <v>397</v>
+        <v>98</v>
+      </c>
+      <c r="K64" s="2" t="n">
+        <v>364</v>
       </c>
     </row>
     <row r="65" ht="60" customHeight="1">
@@ -5150,19 +5499,20 @@
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
+          <t>cloro.png</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
           <t>1 L</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>63</v>
-      </c>
+      <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="2" t="n">
-        <v>203</v>
+        <v>55</v>
+      </c>
+      <c r="K65" s="2" t="n">
+        <v>206</v>
       </c>
     </row>
     <row r="66" ht="60" customHeight="1">
@@ -5194,15 +5544,20 @@
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
+          <t>desinfectante.png</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
           <t>1 L</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr"/>
-      <c r="I66" s="2" t="n">
-        <v>62</v>
-      </c>
+      <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="n">
-        <v>307</v>
+        <v>24</v>
+      </c>
+      <c r="K66" s="2" t="n">
+        <v>321</v>
       </c>
     </row>
     <row r="67" ht="60" customHeight="1">
@@ -5234,15 +5589,20 @@
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
+          <t>esponja.png</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
           <t>3 Unidades</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr"/>
-      <c r="I67" s="2" t="n">
-        <v>84</v>
-      </c>
+      <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="n">
-        <v>231</v>
+        <v>21</v>
+      </c>
+      <c r="K67" s="2" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="68" ht="60" customHeight="1">
@@ -5274,15 +5634,20 @@
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
+          <t>mopa.png</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr"/>
-      <c r="I68" s="2" t="n">
-        <v>45</v>
-      </c>
+      <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="n">
-        <v>402</v>
+        <v>78</v>
+      </c>
+      <c r="K68" s="2" t="n">
+        <v>276</v>
       </c>
     </row>
     <row r="69" ht="60" customHeight="1">
@@ -5314,15 +5679,20 @@
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
+          <t>escoba.png</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr"/>
-      <c r="I69" s="2" t="n">
-        <v>89</v>
-      </c>
+      <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="2" t="n">
-        <v>340</v>
+        <v>47</v>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>323</v>
       </c>
     </row>
     <row r="70" ht="60" customHeight="1">
@@ -5354,15 +5724,20 @@
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
+          <t>coleto.png</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="n">
-        <v>87</v>
-      </c>
+      <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="n">
-        <v>338</v>
+        <v>92</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>161</v>
       </c>
     </row>
     <row r="71" ht="60" customHeight="1">
@@ -5394,15 +5769,24 @@
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
+          <t>bolsas_basura.png</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
           <t>10 Unidades</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr"/>
-      <c r="I71" s="2" t="n">
-        <v>84</v>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J71" s="2" t="n">
-        <v>343</v>
+        <v>100</v>
+      </c>
+      <c r="K71" s="2" t="n">
+        <v>421</v>
       </c>
     </row>
     <row r="72" ht="60" customHeight="1">
@@ -5434,15 +5818,24 @@
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
+          <t>cerveza_pilsen.png</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
           <t>Caja 36</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="2" t="n">
-        <v>84</v>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
       </c>
       <c r="J72" s="2" t="n">
-        <v>275</v>
+        <v>96</v>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>235</v>
       </c>
     </row>
     <row r="73" ht="60" customHeight="1">
@@ -5474,19 +5867,20 @@
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
+          <t>cerveza_light.png</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
           <t>Caja 36</t>
         </is>
       </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="n">
-        <v>71</v>
-      </c>
+      <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="n">
-        <v>138</v>
+        <v>79</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>144</v>
       </c>
     </row>
     <row r="74" ht="60" customHeight="1">
@@ -5518,15 +5912,20 @@
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
+          <t>cerveza_solera.png</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
           <t>6 Pack</t>
         </is>
       </c>
-      <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="n">
-        <v>61</v>
-      </c>
+      <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="n">
-        <v>480</v>
+        <v>15</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>238</v>
       </c>
     </row>
     <row r="75" ht="60" customHeight="1">
@@ -5558,15 +5957,20 @@
       <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
+          <t>cerveza_zulia.png</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
           <t>6 Pack</t>
         </is>
       </c>
-      <c r="H75" s="2" t="inlineStr"/>
-      <c r="I75" s="2" t="n">
-        <v>65</v>
-      </c>
+      <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="n">
-        <v>260</v>
+        <v>33</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>314</v>
       </c>
     </row>
     <row r="76" ht="60" customHeight="1">
@@ -5598,19 +6002,20 @@
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
+          <t>ron_teresa.png</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="n">
-        <v>98</v>
-      </c>
+      <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="n">
-        <v>363</v>
+        <v>14</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>241</v>
       </c>
     </row>
     <row r="77" ht="60" customHeight="1">
@@ -5642,19 +6047,24 @@
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
+          <t>ron_cacique.png</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="I77" s="2" t="inlineStr">
         <is>
           <t>Nuevo</t>
         </is>
       </c>
-      <c r="I77" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="J77" s="2" t="n">
-        <v>347</v>
+        <v>24</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>415</v>
       </c>
     </row>
     <row r="78" ht="60" customHeight="1">
@@ -5686,19 +6096,20 @@
       <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
+          <t>ron_pampero.png</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="n">
-        <v>95</v>
-      </c>
+      <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="n">
-        <v>497</v>
+        <v>29</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>160</v>
       </c>
     </row>
     <row r="79" ht="60" customHeight="1">
@@ -5730,19 +6141,20 @@
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
+          <t>ron_diplomatico.png</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="I79" s="2" t="n">
-        <v>11</v>
-      </c>
+      <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="n">
-        <v>143</v>
+        <v>34</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>338</v>
       </c>
     </row>
     <row r="80" ht="60" customHeight="1">
@@ -5774,15 +6186,20 @@
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
+          <t>whisky_buchanans.png</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr"/>
-      <c r="I80" s="2" t="n">
-        <v>94</v>
-      </c>
+      <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="n">
-        <v>154</v>
+        <v>57</v>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="81" ht="60" customHeight="1">
@@ -5814,15 +6231,24 @@
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
+          <t>whisky_parr.png</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H81" s="2" t="inlineStr"/>
-      <c r="I81" s="2" t="n">
-        <v>17</v>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J81" s="2" t="n">
-        <v>123</v>
+        <v>83</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>313</v>
       </c>
     </row>
     <row r="82" ht="60" customHeight="1">
@@ -5854,19 +6280,24 @@
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
+          <t>vodka.png</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="n">
-        <v>77</v>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J82" s="2" t="n">
-        <v>327</v>
+        <v>58</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>260</v>
       </c>
     </row>
     <row r="83" ht="60" customHeight="1">
@@ -5898,19 +6329,24 @@
       <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
+          <t>vino_tinto.png</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="I83" s="2" t="n">
-        <v>98</v>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
       </c>
       <c r="J83" s="2" t="n">
-        <v>333</v>
+        <v>36</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>81</v>
       </c>
     </row>
     <row r="84" ht="60" customHeight="1">
@@ -5942,15 +6378,20 @@
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
+          <t>vino_blanco.png</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
           <t>750ml</t>
         </is>
       </c>
-      <c r="H84" s="2" t="inlineStr"/>
-      <c r="I84" s="2" t="n">
-        <v>23</v>
-      </c>
+      <c r="I84" s="2" t="inlineStr"/>
       <c r="J84" s="2" t="n">
-        <v>217</v>
+        <v>82</v>
+      </c>
+      <c r="K84" s="2" t="n">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add premium checkout flow, link cart login redirection, and generate/sync refrigerated product images on pure white backgrounds
</commit_message>
<xml_diff>
--- a/frontend/public/data/productos_inventario.xlsx
+++ b/frontend/public/data/productos_inventario.xlsx
@@ -2614,10 +2614,10 @@
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>68</v>
+        <v>362</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
@@ -2659,10 +2659,10 @@
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="n">
-        <v>75</v>
+        <v>12</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>497</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
@@ -2702,16 +2702,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="n">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>276</v>
+        <v>423</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
@@ -2751,12 +2747,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="n">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>276</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
@@ -2798,14 +2798,14 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Oferta</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>477</v>
+        <v>367</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
@@ -2845,16 +2845,12 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="n">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>458</v>
+        <v>341</v>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
@@ -2896,10 +2892,10 @@
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>313</v>
+        <v>351</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
@@ -2941,10 +2937,10 @@
       </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>128</v>
+        <v>462</v>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
@@ -2986,10 +2982,10 @@
       </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>336</v>
+        <v>421</v>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
@@ -3031,10 +3027,10 @@
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>417</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
@@ -3076,10 +3072,10 @@
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>167</v>
+        <v>403</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
@@ -3119,12 +3115,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="n">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>109</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
@@ -3166,10 +3166,10 @@
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="n">
-        <v>38</v>
+        <v>93</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>340</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
@@ -3209,12 +3209,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>486</v>
+        <v>462</v>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
@@ -3254,16 +3258,12 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="n">
-        <v>30</v>
+        <v>68</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>384</v>
+        <v>395</v>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
@@ -3305,10 +3305,10 @@
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>271</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
@@ -3348,12 +3348,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="n">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>399</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
@@ -3395,10 +3399,10 @@
       </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>253</v>
+        <v>362</v>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
@@ -3440,10 +3444,10 @@
       </c>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>158</v>
+        <v>382</v>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
@@ -3485,10 +3489,10 @@
       </c>
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="n">
-        <v>90</v>
+        <v>12</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>285</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
@@ -3530,10 +3534,10 @@
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>472</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
@@ -3573,16 +3577,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>287</v>
+        <v>205</v>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1">
@@ -3624,10 +3624,10 @@
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>454</v>
+        <v>335</v>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -3669,10 +3669,10 @@
       </c>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="n">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>419</v>
+        <v>341</v>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
@@ -3714,10 +3714,10 @@
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>457</v>
+        <v>303</v>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
@@ -3759,10 +3759,10 @@
       </c>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>296</v>
+        <v>451</v>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
@@ -3802,16 +3802,12 @@
           <t>250g</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="n">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>162</v>
+        <v>454</v>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
@@ -3851,12 +3847,16 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="n">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>157</v>
+        <v>453</v>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
@@ -3898,10 +3898,10 @@
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="n">
-        <v>47</v>
+        <v>82</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>220</v>
+        <v>256</v>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
@@ -3943,10 +3943,10 @@
       </c>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="n">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>95</v>
+        <v>249</v>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
@@ -3986,16 +3986,12 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="n">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>309</v>
+        <v>273</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -4037,10 +4033,10 @@
       </c>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>427</v>
+        <v>404</v>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
@@ -4082,10 +4078,10 @@
       </c>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>193</v>
+        <v>375</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
@@ -4125,16 +4121,12 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="n">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>446</v>
+        <v>261</v>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
@@ -4174,16 +4166,12 @@
           <t>1.5 L</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="n">
-        <v>19</v>
+        <v>87</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>257</v>
+        <v>232</v>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
@@ -4225,10 +4213,10 @@
       </c>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="n">
-        <v>86</v>
+        <v>21</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>294</v>
+        <v>304</v>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
@@ -4270,10 +4258,10 @@
       </c>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>443</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
@@ -4313,16 +4301,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="n">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>72</v>
+        <v>500</v>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
@@ -4362,12 +4346,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="n">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>96</v>
+        <v>431</v>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
@@ -4409,10 +4397,10 @@
       </c>
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="n">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>149</v>
+        <v>298</v>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
@@ -4454,10 +4442,10 @@
       </c>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="n">
-        <v>74</v>
+        <v>16</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>197</v>
+        <v>316</v>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
@@ -4497,12 +4485,16 @@
           <t>140g</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J43" s="2" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>162</v>
+        <v>262</v>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
@@ -4544,10 +4536,10 @@
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="n">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>78</v>
+        <v>339</v>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
@@ -4589,10 +4581,10 @@
       </c>
       <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>193</v>
+        <v>242</v>
       </c>
     </row>
     <row r="46" ht="60" customHeight="1">
@@ -4632,12 +4624,16 @@
           <t>1 Litro</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J46" s="2" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>237</v>
+        <v>70</v>
       </c>
     </row>
     <row r="47" ht="60" customHeight="1">
@@ -4677,16 +4673,12 @@
           <t>3 Unidades</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>302</v>
+        <v>99</v>
       </c>
     </row>
     <row r="48" ht="60" customHeight="1">
@@ -4728,14 +4720,14 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Oferta</t>
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
@@ -4777,10 +4769,10 @@
       </c>
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="n">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>108</v>
+        <v>479</v>
       </c>
     </row>
     <row r="50" ht="60" customHeight="1">
@@ -4820,12 +4812,16 @@
           <t>400ml</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="n">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>55</v>
+        <v>437</v>
       </c>
     </row>
     <row r="51" ht="60" customHeight="1">
@@ -4867,10 +4863,10 @@
       </c>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="n">
-        <v>81</v>
+        <v>31</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>372</v>
+        <v>381</v>
       </c>
     </row>
     <row r="52" ht="60" customHeight="1">
@@ -4912,10 +4908,10 @@
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="n">
-        <v>92</v>
+        <v>13</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53" ht="60" customHeight="1">
@@ -4957,10 +4953,10 @@
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>312</v>
+        <v>146</v>
       </c>
     </row>
     <row r="54" ht="60" customHeight="1">
@@ -5002,10 +4998,10 @@
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>189</v>
+        <v>470</v>
       </c>
     </row>
     <row r="55" ht="60" customHeight="1">
@@ -5047,10 +5043,10 @@
       </c>
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="n">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>192</v>
+        <v>237</v>
       </c>
     </row>
     <row r="56" ht="60" customHeight="1">
@@ -5090,16 +5086,12 @@
           <t>100 Unidades</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>55</v>
+        <v>223</v>
       </c>
     </row>
     <row r="57" ht="60" customHeight="1">
@@ -5139,12 +5131,16 @@
           <t>250ml</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J57" s="2" t="n">
-        <v>45</v>
+        <v>98</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>372</v>
+        <v>187</v>
       </c>
     </row>
     <row r="58" ht="60" customHeight="1">
@@ -5184,16 +5180,12 @@
           <t>100ml</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="n">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>284</v>
+        <v>474</v>
       </c>
     </row>
     <row r="59" ht="60" customHeight="1">
@@ -5235,10 +5227,10 @@
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="n">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>341</v>
+        <v>454</v>
       </c>
     </row>
     <row r="60" ht="60" customHeight="1">
@@ -5278,12 +5270,16 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J60" s="2" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>131</v>
+        <v>62</v>
       </c>
     </row>
     <row r="61" ht="60" customHeight="1">
@@ -5323,12 +5319,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J61" s="2" t="n">
-        <v>90</v>
+        <v>54</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>313</v>
+        <v>180</v>
       </c>
     </row>
     <row r="62" ht="60" customHeight="1">
@@ -5368,16 +5368,12 @@
           <t>1 L</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="n">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>446</v>
+        <v>263</v>
       </c>
     </row>
     <row r="63" ht="60" customHeight="1">
@@ -5419,10 +5415,10 @@
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="n">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>363</v>
+        <v>79</v>
       </c>
     </row>
     <row r="64" ht="60" customHeight="1">
@@ -5464,10 +5460,10 @@
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="n">
-        <v>11</v>
+        <v>94</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>427</v>
+        <v>180</v>
       </c>
     </row>
     <row r="65" ht="60" customHeight="1">
@@ -5507,12 +5503,16 @@
           <t>1 L</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>272</v>
+        <v>481</v>
       </c>
     </row>
     <row r="66" ht="60" customHeight="1">
@@ -5554,10 +5554,10 @@
       </c>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="n">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>435</v>
+        <v>251</v>
       </c>
     </row>
     <row r="67" ht="60" customHeight="1">
@@ -5597,16 +5597,12 @@
           <t>3 Unidades</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>456</v>
+        <v>126</v>
       </c>
     </row>
     <row r="68" ht="60" customHeight="1">
@@ -5648,10 +5644,10 @@
       </c>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>137</v>
+        <v>208</v>
       </c>
     </row>
     <row r="69" ht="60" customHeight="1">
@@ -5691,12 +5687,16 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J69" s="2" t="n">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>328</v>
+        <v>477</v>
       </c>
     </row>
     <row r="70" ht="60" customHeight="1">
@@ -5738,10 +5738,10 @@
       </c>
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="n">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>288</v>
+        <v>492</v>
       </c>
     </row>
     <row r="71" ht="60" customHeight="1">
@@ -5783,10 +5783,10 @@
       </c>
       <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>208</v>
+        <v>490</v>
       </c>
     </row>
     <row r="72" ht="60" customHeight="1">
@@ -5828,10 +5828,10 @@
       </c>
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>102</v>
+        <v>143</v>
       </c>
     </row>
     <row r="73" ht="60" customHeight="1">
@@ -5873,10 +5873,10 @@
       </c>
       <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="n">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>492</v>
+        <v>436</v>
       </c>
     </row>
     <row r="74" ht="60" customHeight="1">
@@ -5916,16 +5916,12 @@
           <t>6 Pack</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>50</v>
+        <v>324</v>
       </c>
     </row>
     <row r="75" ht="60" customHeight="1">
@@ -5967,10 +5963,10 @@
       </c>
       <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="n">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>73</v>
+        <v>191</v>
       </c>
     </row>
     <row r="76" ht="60" customHeight="1">
@@ -6012,10 +6008,10 @@
       </c>
       <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="n">
-        <v>81</v>
+        <v>32</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>392</v>
+        <v>245</v>
       </c>
     </row>
     <row r="77" ht="60" customHeight="1">
@@ -6057,10 +6053,10 @@
       </c>
       <c r="I77" s="2" t="inlineStr"/>
       <c r="J77" s="2" t="n">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>366</v>
+        <v>190</v>
       </c>
     </row>
     <row r="78" ht="60" customHeight="1">
@@ -6100,12 +6096,16 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J78" s="2" t="n">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>334</v>
+        <v>163</v>
       </c>
     </row>
     <row r="79" ht="60" customHeight="1">
@@ -6147,10 +6147,10 @@
       </c>
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="n">
-        <v>25</v>
+        <v>94</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>50</v>
+        <v>102</v>
       </c>
     </row>
     <row r="80" ht="60" customHeight="1">
@@ -6192,10 +6192,10 @@
       </c>
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>170</v>
+        <v>451</v>
       </c>
     </row>
     <row r="81" ht="60" customHeight="1">
@@ -6237,14 +6237,14 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Oferta</t>
         </is>
       </c>
       <c r="J81" s="2" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>274</v>
+        <v>371</v>
       </c>
     </row>
     <row r="82" ht="60" customHeight="1">
@@ -6286,10 +6286,10 @@
       </c>
       <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="n">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>52</v>
+        <v>74</v>
       </c>
     </row>
     <row r="83" ht="60" customHeight="1">
@@ -6329,16 +6329,12 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I83" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I83" s="2" t="inlineStr"/>
       <c r="J83" s="2" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>498</v>
+        <v>207</v>
       </c>
     </row>
     <row r="84" ht="60" customHeight="1">
@@ -6378,16 +6374,12 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I84" s="2" t="inlineStr"/>
       <c r="J84" s="2" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>402</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update first 3 products of Víveres (coca_cola, pepsi, chinotto) with new pure-white-background images, and compile to database
</commit_message>
<xml_diff>
--- a/frontend/public/data/productos_inventario.xlsx
+++ b/frontend/public/data/productos_inventario.xlsx
@@ -2614,10 +2614,10 @@
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>362</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
@@ -2657,12 +2657,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>316</v>
+        <v>454</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
@@ -2702,12 +2706,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="n">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>423</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
@@ -2753,10 +2761,10 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>210</v>
+        <v>458</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
@@ -2796,16 +2804,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="n">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>367</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
@@ -2847,10 +2851,10 @@
       </c>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>341</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
@@ -2892,10 +2896,10 @@
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>351</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
@@ -2937,10 +2941,10 @@
       </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>462</v>
+        <v>498</v>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
@@ -2982,10 +2986,10 @@
       </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>421</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
@@ -3027,10 +3031,10 @@
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>171</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
@@ -3072,10 +3076,10 @@
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="n">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>403</v>
+        <v>352</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
@@ -3115,16 +3119,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="n">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>236</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
@@ -3166,10 +3166,10 @@
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="n">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>251</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
@@ -3209,16 +3209,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>462</v>
+        <v>410</v>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
@@ -3260,10 +3256,10 @@
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>395</v>
+        <v>490</v>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
@@ -3305,10 +3301,10 @@
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="n">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>111</v>
+        <v>403</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
@@ -3348,16 +3344,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="n">
-        <v>86</v>
+        <v>34</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>235</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
@@ -3399,10 +3391,10 @@
       </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>362</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
@@ -3444,10 +3436,10 @@
       </c>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="n">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>382</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
@@ -3489,10 +3481,10 @@
       </c>
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>81</v>
+        <v>496</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
@@ -3534,10 +3526,10 @@
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n">
-        <v>99</v>
+        <v>41</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>92</v>
+        <v>465</v>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
@@ -3579,10 +3571,10 @@
       </c>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="n">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>205</v>
+        <v>287</v>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1">
@@ -3624,10 +3616,10 @@
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>335</v>
+        <v>265</v>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -3667,12 +3659,16 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="n">
-        <v>22</v>
+        <v>98</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>341</v>
+        <v>442</v>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
@@ -3714,10 +3710,10 @@
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>303</v>
+        <v>401</v>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
@@ -3759,10 +3755,10 @@
       </c>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>451</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
@@ -3802,12 +3798,16 @@
           <t>250g</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>454</v>
+        <v>387</v>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
@@ -3847,16 +3847,12 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="n">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>453</v>
+        <v>434</v>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
@@ -3898,10 +3894,10 @@
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="n">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>256</v>
+        <v>355</v>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
@@ -3943,10 +3939,10 @@
       </c>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="n">
-        <v>89</v>
+        <v>55</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>249</v>
+        <v>215</v>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
@@ -3988,10 +3984,10 @@
       </c>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>273</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -4033,10 +4029,10 @@
       </c>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="n">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>404</v>
+        <v>411</v>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
@@ -4078,10 +4074,10 @@
       </c>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="n">
-        <v>88</v>
+        <v>46</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>375</v>
+        <v>429</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
@@ -4123,10 +4119,10 @@
       </c>
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="n">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>261</v>
+        <v>185</v>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
@@ -4168,10 +4164,10 @@
       </c>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="n">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>232</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
@@ -4213,10 +4209,10 @@
       </c>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>304</v>
+        <v>158</v>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
@@ -4258,10 +4254,10 @@
       </c>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="n">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>148</v>
+        <v>430</v>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
@@ -4303,10 +4299,10 @@
       </c>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="n">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>500</v>
+        <v>102</v>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
@@ -4346,16 +4342,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="n">
-        <v>10</v>
+        <v>81</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>431</v>
+        <v>379</v>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
@@ -4397,10 +4389,10 @@
       </c>
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>298</v>
+        <v>203</v>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
@@ -4442,10 +4434,10 @@
       </c>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="n">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>316</v>
+        <v>416</v>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
@@ -4485,16 +4477,12 @@
           <t>140g</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>262</v>
+        <v>225</v>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
@@ -4536,10 +4524,10 @@
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="n">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>339</v>
+        <v>351</v>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
@@ -4579,12 +4567,16 @@
           <t>300g</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J45" s="2" t="n">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>242</v>
+        <v>204</v>
       </c>
     </row>
     <row r="46" ht="60" customHeight="1">
@@ -4624,16 +4616,12 @@
           <t>1 Litro</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="n">
-        <v>99</v>
+        <v>42</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>70</v>
+        <v>307</v>
       </c>
     </row>
     <row r="47" ht="60" customHeight="1">
@@ -4675,10 +4663,10 @@
       </c>
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="n">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>99</v>
+        <v>269</v>
       </c>
     </row>
     <row r="48" ht="60" customHeight="1">
@@ -4718,16 +4706,12 @@
           <t>50ml</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>360</v>
+        <v>242</v>
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
@@ -4767,12 +4751,16 @@
           <t>100g</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J49" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>479</v>
+        <v>133</v>
       </c>
     </row>
     <row r="50" ht="60" customHeight="1">
@@ -4812,13 +4800,9 @@
           <t>400ml</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="n">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>437</v>
@@ -4863,10 +4847,10 @@
       </c>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>381</v>
+        <v>450</v>
       </c>
     </row>
     <row r="52" ht="60" customHeight="1">
@@ -4908,10 +4892,10 @@
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="n">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>119</v>
+        <v>196</v>
       </c>
     </row>
     <row r="53" ht="60" customHeight="1">
@@ -4953,10 +4937,10 @@
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>146</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" ht="60" customHeight="1">
@@ -4998,10 +4982,10 @@
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>470</v>
+        <v>351</v>
       </c>
     </row>
     <row r="55" ht="60" customHeight="1">
@@ -5043,10 +5027,10 @@
       </c>
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="n">
-        <v>99</v>
+        <v>48</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>237</v>
+        <v>192</v>
       </c>
     </row>
     <row r="56" ht="60" customHeight="1">
@@ -5088,10 +5072,10 @@
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="n">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>223</v>
+        <v>377</v>
       </c>
     </row>
     <row r="57" ht="60" customHeight="1">
@@ -5131,16 +5115,12 @@
           <t>250ml</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="n">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>187</v>
+        <v>357</v>
       </c>
     </row>
     <row r="58" ht="60" customHeight="1">
@@ -5180,12 +5160,16 @@
           <t>100ml</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="n">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>474</v>
+        <v>380</v>
       </c>
     </row>
     <row r="59" ht="60" customHeight="1">
@@ -5227,10 +5211,10 @@
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>454</v>
+        <v>387</v>
       </c>
     </row>
     <row r="60" ht="60" customHeight="1">
@@ -5270,16 +5254,12 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="n">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>62</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" ht="60" customHeight="1">
@@ -5319,16 +5299,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I61" s="2" t="inlineStr"/>
       <c r="J61" s="2" t="n">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>180</v>
+        <v>83</v>
       </c>
     </row>
     <row r="62" ht="60" customHeight="1">
@@ -5368,12 +5344,16 @@
           <t>1 L</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J62" s="2" t="n">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>263</v>
+        <v>176</v>
       </c>
     </row>
     <row r="63" ht="60" customHeight="1">
@@ -5415,10 +5395,10 @@
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="n">
-        <v>92</v>
+        <v>29</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>79</v>
+        <v>423</v>
       </c>
     </row>
     <row r="64" ht="60" customHeight="1">
@@ -5460,10 +5440,10 @@
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>180</v>
+        <v>327</v>
       </c>
     </row>
     <row r="65" ht="60" customHeight="1">
@@ -5503,16 +5483,12 @@
           <t>1 L</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="2" t="n">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>481</v>
+        <v>277</v>
       </c>
     </row>
     <row r="66" ht="60" customHeight="1">
@@ -5554,10 +5530,10 @@
       </c>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="n">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>251</v>
+        <v>401</v>
       </c>
     </row>
     <row r="67" ht="60" customHeight="1">
@@ -5599,10 +5575,10 @@
       </c>
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="n">
-        <v>31</v>
+        <v>91</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>126</v>
+        <v>300</v>
       </c>
     </row>
     <row r="68" ht="60" customHeight="1">
@@ -5644,10 +5620,10 @@
       </c>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>208</v>
+        <v>422</v>
       </c>
     </row>
     <row r="69" ht="60" customHeight="1">
@@ -5687,16 +5663,12 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="2" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>477</v>
+        <v>237</v>
       </c>
     </row>
     <row r="70" ht="60" customHeight="1">
@@ -5736,12 +5708,16 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J70" s="2" t="n">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>492</v>
+        <v>255</v>
       </c>
     </row>
     <row r="71" ht="60" customHeight="1">
@@ -5783,10 +5759,10 @@
       </c>
       <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>490</v>
+        <v>402</v>
       </c>
     </row>
     <row r="72" ht="60" customHeight="1">
@@ -5828,10 +5804,10 @@
       </c>
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="n">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>143</v>
+        <v>386</v>
       </c>
     </row>
     <row r="73" ht="60" customHeight="1">
@@ -5871,12 +5847,16 @@
           <t>Caja 36</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J73" s="2" t="n">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>436</v>
+        <v>495</v>
       </c>
     </row>
     <row r="74" ht="60" customHeight="1">
@@ -5918,10 +5898,10 @@
       </c>
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>324</v>
+        <v>497</v>
       </c>
     </row>
     <row r="75" ht="60" customHeight="1">
@@ -5963,10 +5943,10 @@
       </c>
       <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="n">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>191</v>
+        <v>168</v>
       </c>
     </row>
     <row r="76" ht="60" customHeight="1">
@@ -6006,12 +5986,16 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J76" s="2" t="n">
-        <v>32</v>
+        <v>89</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>245</v>
+        <v>477</v>
       </c>
     </row>
     <row r="77" ht="60" customHeight="1">
@@ -6053,10 +6037,10 @@
       </c>
       <c r="I77" s="2" t="inlineStr"/>
       <c r="J77" s="2" t="n">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>190</v>
+        <v>153</v>
       </c>
     </row>
     <row r="78" ht="60" customHeight="1">
@@ -6102,10 +6086,10 @@
         </is>
       </c>
       <c r="J78" s="2" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>163</v>
+        <v>471</v>
       </c>
     </row>
     <row r="79" ht="60" customHeight="1">
@@ -6147,10 +6131,10 @@
       </c>
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="n">
-        <v>94</v>
+        <v>16</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="80" ht="60" customHeight="1">
@@ -6192,10 +6176,10 @@
       </c>
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>451</v>
+        <v>169</v>
       </c>
     </row>
     <row r="81" ht="60" customHeight="1">
@@ -6235,16 +6219,12 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I81" s="2" t="inlineStr"/>
       <c r="J81" s="2" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>371</v>
+        <v>229</v>
       </c>
     </row>
     <row r="82" ht="60" customHeight="1">
@@ -6286,10 +6266,10 @@
       </c>
       <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>74</v>
+        <v>194</v>
       </c>
     </row>
     <row r="83" ht="60" customHeight="1">
@@ -6331,10 +6311,10 @@
       </c>
       <c r="I83" s="2" t="inlineStr"/>
       <c r="J83" s="2" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>207</v>
+        <v>431</v>
       </c>
     </row>
     <row r="84" ht="60" customHeight="1">
@@ -6374,12 +6354,16 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J84" s="2" t="n">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>55</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Batch 2 of Víveres with high-quality 10-step images and sync to database
</commit_message>
<xml_diff>
--- a/frontend/public/data/productos_inventario.xlsx
+++ b/frontend/public/data/productos_inventario.xlsx
@@ -2612,12 +2612,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="n">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>206</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
@@ -2657,16 +2661,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>454</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
@@ -2712,10 +2712,10 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>350</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
@@ -2755,16 +2755,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>458</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
@@ -2806,10 +2802,10 @@
       </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="n">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>357</v>
+        <v>404</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
@@ -2851,10 +2847,10 @@
       </c>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>306</v>
+        <v>348</v>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
@@ -2896,7 +2892,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>189</v>
@@ -2941,10 +2937,10 @@
       </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>498</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
@@ -2986,10 +2982,10 @@
       </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>284</v>
+        <v>306</v>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
@@ -3029,12 +3025,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="n">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>73</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
@@ -3074,12 +3074,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="n">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>352</v>
+        <v>324</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
@@ -3119,12 +3123,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="n">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>72</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
@@ -3166,10 +3174,10 @@
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="n">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
@@ -3211,10 +3219,10 @@
       </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="n">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>410</v>
+        <v>173</v>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
@@ -3256,10 +3264,10 @@
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="n">
-        <v>62</v>
+        <v>96</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>490</v>
+        <v>359</v>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
@@ -3301,10 +3309,10 @@
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="n">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>403</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
@@ -3344,12 +3352,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="n">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>120</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
@@ -3391,10 +3403,10 @@
       </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>136</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
@@ -3436,7 +3448,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="n">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>71</v>
@@ -3479,12 +3491,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>496</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
@@ -3526,10 +3542,10 @@
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>465</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
@@ -3571,10 +3587,10 @@
       </c>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="n">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>287</v>
+        <v>298</v>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1">
@@ -3616,10 +3632,10 @@
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="n">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>265</v>
+        <v>323</v>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -3659,16 +3675,12 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="n">
         <v>98</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>442</v>
+        <v>460</v>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
@@ -3710,10 +3722,10 @@
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="n">
-        <v>15</v>
+        <v>84</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>401</v>
+        <v>282</v>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
@@ -3755,10 +3767,10 @@
       </c>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>82</v>
+        <v>430</v>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
@@ -3798,16 +3810,12 @@
           <t>250g</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>387</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
@@ -3849,10 +3857,10 @@
       </c>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>434</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
@@ -3894,10 +3902,10 @@
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="n">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>355</v>
+        <v>496</v>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
@@ -3939,10 +3947,10 @@
       </c>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>215</v>
+        <v>322</v>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
@@ -3984,10 +3992,10 @@
       </c>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>200</v>
+        <v>225</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -4029,10 +4037,10 @@
       </c>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>411</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
@@ -4074,10 +4082,10 @@
       </c>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="n">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>429</v>
+        <v>173</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
@@ -4119,10 +4127,10 @@
       </c>
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="n">
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>185</v>
+        <v>279</v>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
@@ -4162,12 +4170,16 @@
           <t>1.5 L</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="n">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>59</v>
+        <v>482</v>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
@@ -4209,10 +4221,10 @@
       </c>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="n">
-        <v>14</v>
+        <v>94</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>158</v>
+        <v>443</v>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
@@ -4254,10 +4266,10 @@
       </c>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
@@ -4299,10 +4311,10 @@
       </c>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="n">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>102</v>
+        <v>327</v>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
@@ -4342,12 +4354,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="n">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>379</v>
+        <v>331</v>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
@@ -4389,10 +4405,10 @@
       </c>
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="n">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>203</v>
+        <v>461</v>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
@@ -4434,10 +4450,10 @@
       </c>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>416</v>
+        <v>174</v>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
@@ -4479,10 +4495,10 @@
       </c>
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="n">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
@@ -4524,10 +4540,10 @@
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>351</v>
+        <v>218</v>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
@@ -4567,16 +4583,12 @@
           <t>300g</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>204</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" ht="60" customHeight="1">
@@ -4618,10 +4630,10 @@
       </c>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="n">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>307</v>
+        <v>193</v>
       </c>
     </row>
     <row r="47" ht="60" customHeight="1">
@@ -4663,10 +4675,10 @@
       </c>
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="n">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>269</v>
+        <v>82</v>
       </c>
     </row>
     <row r="48" ht="60" customHeight="1">
@@ -4708,10 +4720,10 @@
       </c>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="n">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
@@ -4751,16 +4763,12 @@
           <t>100g</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>133</v>
+        <v>284</v>
       </c>
     </row>
     <row r="50" ht="60" customHeight="1">
@@ -4800,12 +4808,16 @@
           <t>400ml</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="n">
         <v>56</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>437</v>
+        <v>492</v>
       </c>
     </row>
     <row r="51" ht="60" customHeight="1">
@@ -4847,10 +4859,10 @@
       </c>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>450</v>
+        <v>192</v>
       </c>
     </row>
     <row r="52" ht="60" customHeight="1">
@@ -4892,10 +4904,10 @@
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="n">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>196</v>
+        <v>361</v>
       </c>
     </row>
     <row r="53" ht="60" customHeight="1">
@@ -4937,10 +4949,10 @@
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="n">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>97</v>
+        <v>401</v>
       </c>
     </row>
     <row r="54" ht="60" customHeight="1">
@@ -4982,10 +4994,10 @@
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="n">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>351</v>
+        <v>72</v>
       </c>
     </row>
     <row r="55" ht="60" customHeight="1">
@@ -5027,10 +5039,10 @@
       </c>
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="n">
-        <v>48</v>
+        <v>94</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>192</v>
+        <v>349</v>
       </c>
     </row>
     <row r="56" ht="60" customHeight="1">
@@ -5072,10 +5084,10 @@
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>377</v>
+        <v>500</v>
       </c>
     </row>
     <row r="57" ht="60" customHeight="1">
@@ -5117,10 +5129,10 @@
       </c>
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>357</v>
+        <v>346</v>
       </c>
     </row>
     <row r="58" ht="60" customHeight="1">
@@ -5160,16 +5172,12 @@
           <t>100ml</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="n">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>380</v>
+        <v>257</v>
       </c>
     </row>
     <row r="59" ht="60" customHeight="1">
@@ -5211,10 +5219,10 @@
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>387</v>
+        <v>319</v>
       </c>
     </row>
     <row r="60" ht="60" customHeight="1">
@@ -5256,10 +5264,10 @@
       </c>
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="n">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>135</v>
+        <v>446</v>
       </c>
     </row>
     <row r="61" ht="60" customHeight="1">
@@ -5299,12 +5307,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J61" s="2" t="n">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>83</v>
+        <v>155</v>
       </c>
     </row>
     <row r="62" ht="60" customHeight="1">
@@ -5344,16 +5356,12 @@
           <t>1 L</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>176</v>
+        <v>460</v>
       </c>
     </row>
     <row r="63" ht="60" customHeight="1">
@@ -5395,10 +5403,10 @@
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="n">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>423</v>
+        <v>284</v>
       </c>
     </row>
     <row r="64" ht="60" customHeight="1">
@@ -5440,10 +5448,10 @@
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="n">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>327</v>
+        <v>499</v>
       </c>
     </row>
     <row r="65" ht="60" customHeight="1">
@@ -5483,12 +5491,16 @@
           <t>1 L</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="n">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>277</v>
+        <v>50</v>
       </c>
     </row>
     <row r="66" ht="60" customHeight="1">
@@ -5530,10 +5542,10 @@
       </c>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>401</v>
+        <v>271</v>
       </c>
     </row>
     <row r="67" ht="60" customHeight="1">
@@ -5573,12 +5585,16 @@
           <t>3 Unidades</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J67" s="2" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>300</v>
+        <v>148</v>
       </c>
     </row>
     <row r="68" ht="60" customHeight="1">
@@ -5620,10 +5636,10 @@
       </c>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="n">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>422</v>
+        <v>472</v>
       </c>
     </row>
     <row r="69" ht="60" customHeight="1">
@@ -5665,10 +5681,10 @@
       </c>
       <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="2" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>237</v>
+        <v>455</v>
       </c>
     </row>
     <row r="70" ht="60" customHeight="1">
@@ -5708,16 +5724,12 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="n">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>255</v>
+        <v>297</v>
       </c>
     </row>
     <row r="71" ht="60" customHeight="1">
@@ -5759,10 +5771,10 @@
       </c>
       <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>402</v>
+        <v>125</v>
       </c>
     </row>
     <row r="72" ht="60" customHeight="1">
@@ -5804,10 +5816,10 @@
       </c>
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>386</v>
+        <v>256</v>
       </c>
     </row>
     <row r="73" ht="60" customHeight="1">
@@ -5847,13 +5859,9 @@
           <t>Caja 36</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>495</v>
@@ -5898,10 +5906,10 @@
       </c>
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>497</v>
+        <v>298</v>
       </c>
     </row>
     <row r="75" ht="60" customHeight="1">
@@ -5943,10 +5951,10 @@
       </c>
       <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="n">
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>168</v>
+        <v>78</v>
       </c>
     </row>
     <row r="76" ht="60" customHeight="1">
@@ -5986,16 +5994,12 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>477</v>
+        <v>304</v>
       </c>
     </row>
     <row r="77" ht="60" customHeight="1">
@@ -6035,12 +6039,16 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J77" s="2" t="n">
-        <v>23</v>
+        <v>89</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>153</v>
+        <v>128</v>
       </c>
     </row>
     <row r="78" ht="60" customHeight="1">
@@ -6082,14 +6090,14 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Oferta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="J78" s="2" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>471</v>
+        <v>338</v>
       </c>
     </row>
     <row r="79" ht="60" customHeight="1">
@@ -6131,10 +6139,10 @@
       </c>
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>72</v>
+        <v>444</v>
       </c>
     </row>
     <row r="80" ht="60" customHeight="1">
@@ -6176,10 +6184,10 @@
       </c>
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="n">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>169</v>
+        <v>370</v>
       </c>
     </row>
     <row r="81" ht="60" customHeight="1">
@@ -6219,12 +6227,16 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J81" s="2" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>229</v>
+        <v>393</v>
       </c>
     </row>
     <row r="82" ht="60" customHeight="1">
@@ -6264,12 +6276,16 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J82" s="2" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>194</v>
+        <v>484</v>
       </c>
     </row>
     <row r="83" ht="60" customHeight="1">
@@ -6311,10 +6327,10 @@
       </c>
       <c r="I83" s="2" t="inlineStr"/>
       <c r="J83" s="2" t="n">
-        <v>88</v>
+        <v>26</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>431</v>
+        <v>253</v>
       </c>
     </row>
     <row r="84" ht="60" customHeight="1">
@@ -6354,16 +6370,12 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I84" s="2" t="inlineStr"/>
       <c r="J84" s="2" t="n">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>149</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>